<commit_message>
Added new RDF data schemes and visual schemes, and fixed xlsx-spreadsheets for economy-table25-29
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/economy-table26.xlsx
+++ b/sources/table_normalization/xlsx/economy-table26.xlsx
@@ -9891,13 +9891,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF92D050"/>
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor rgb="FF00B050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -9980,31 +9980,31 @@
       <alignment readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
@@ -10308,10 +10308,10 @@
       </c>
     </row>
     <row r="6" spans="2:18" ht="30" customHeight="1">
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="16" t="s">
+      <c r="C6" s="15" t="s">
         <v>4</v>
       </c>
       <c r="D6" s="14" t="s">
@@ -10361,60 +10361,60 @@
       </c>
     </row>
     <row r="7" spans="2:18" ht="30" customHeight="1">
-      <c r="B7" s="15" t="s">
+      <c r="B7" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="15" t="s">
+      <c r="C7" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="12" t="s">
+      <c r="D7" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="12" t="s">
+      <c r="E7" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="F7" s="12" t="s">
+      <c r="F7" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="G7" s="12" t="s">
+      <c r="G7" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="H7" s="12" t="s">
+      <c r="H7" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="I7" s="12" t="s">
+      <c r="I7" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="J7" s="12" t="s">
+      <c r="J7" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="K7" s="12" t="s">
+      <c r="K7" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="L7" s="12" t="s">
+      <c r="L7" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="M7" s="12" t="s">
+      <c r="M7" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="N7" s="12" t="s">
+      <c r="N7" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="O7" s="12" t="s">
+      <c r="O7" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="P7" s="12" t="s">
+      <c r="P7" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="Q7" s="12" t="s">
+      <c r="Q7" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="R7" s="12" t="s">
+      <c r="R7" s="16" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="8" spans="2:18">
-      <c r="B8" s="13" t="s">
+      <c r="B8" s="12" t="s">
         <v>14</v>
       </c>
       <c r="C8" s="1" t="s">
@@ -10485,7 +10485,7 @@
       <c r="O9" s="18"/>
       <c r="P9" s="18"/>
       <c r="Q9" s="18"/>
-      <c r="R9" s="19" t="s">
+      <c r="R9" s="13" t="s">
         <v>15</v>
       </c>
     </row>
@@ -14942,7 +14942,7 @@
       </c>
     </row>
     <row r="94" spans="2:18" ht="15" customHeight="1">
-      <c r="B94" s="20" t="s">
+      <c r="B94" s="19" t="s">
         <v>101</v>
       </c>
       <c r="C94" s="18"/>
@@ -14960,7 +14960,7 @@
       <c r="O94" s="18"/>
       <c r="P94" s="18"/>
       <c r="Q94" s="18"/>
-      <c r="R94" s="19" t="s">
+      <c r="R94" s="13" t="s">
         <v>15</v>
       </c>
     </row>
@@ -19947,7 +19947,7 @@
       </c>
     </row>
     <row r="189" spans="2:18" ht="15" customHeight="1">
-      <c r="B189" s="20" t="s">
+      <c r="B189" s="19" t="s">
         <v>115</v>
       </c>
       <c r="C189" s="18"/>
@@ -19965,7 +19965,7 @@
       <c r="O189" s="18"/>
       <c r="P189" s="18"/>
       <c r="Q189" s="18"/>
-      <c r="R189" s="19" t="s">
+      <c r="R189" s="13" t="s">
         <v>15</v>
       </c>
     </row>
@@ -24952,7 +24952,7 @@
       </c>
     </row>
     <row r="284" spans="2:18" ht="15" customHeight="1">
-      <c r="B284" s="20" t="s">
+      <c r="B284" s="19" t="s">
         <v>119</v>
       </c>
       <c r="C284" s="18"/>
@@ -24970,7 +24970,7 @@
       <c r="O284" s="18"/>
       <c r="P284" s="18"/>
       <c r="Q284" s="18"/>
-      <c r="R284" s="19" t="s">
+      <c r="R284" s="13" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>